<commit_message>
(refactor) Use existing tabs and columns of the metadata workbook for tests
No new tab or column for MSF: tests on a question go in the existing
Comments column as "Test: <what I do> -> <what I should see>", and
scenarios across questions or forms go in the existing, empty "User flow
template" tab (Action = what I do, Description = what I should see,
Step prefixed with the form code). The template is rebuilt from those
existing tabs only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U6uYJ2YYNCsnP72DpH3o5o
</commit_message>
<xml_diff>
--- a/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
+++ b/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
@@ -7,13 +7,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F17-Surgery Admission" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenarios" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User flow template" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form QA Tracker" sheetId="3" state="hidden" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form Guidance" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'F17-Surgery Admission'!$A$2:$BR$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Scenarios'!$A$2:$G$500</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'F17-Surgery Admission'!$A$2:$BP$17</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="[$-2000401]0"/>
     <numFmt numFmtId="166" formatCode="[$-2000000]\d\d\-mmm"/>
   </numFmts>
-  <fonts count="130">
+  <fonts count="129">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -877,11 +876,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="FF2E75B6"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="FF2E75B6"/>
     </font>
@@ -890,7 +884,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="64">
+  <fills count="63">
     <fill>
       <patternFill/>
     </fill>
@@ -1261,11 +1255,6 @@
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF2E75B6"/>
       </patternFill>
     </fill>
   </fills>
@@ -2112,7 +2101,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="804">
+  <cellXfs count="801">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3710,14 +3699,9 @@
     <xf numFmtId="0" fontId="90" fillId="52" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="127" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="63" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="128" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="127" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="129" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="128" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="4">
@@ -8329,9 +8313,9 @@
     <author>LIME</author>
   </authors>
   <commentList>
-    <comment ref="BQ2" authorId="0" shapeId="0">
+    <comment ref="BK2" authorId="0" shapeId="0">
       <text>
-        <t>Optional. One test per row, written as 'If I do... / I should see...'. Skip logic, Mandatory and Lower/Upper limit are already turned into tests automatically: no need to repeat them here.</t>
+        <t>Tests on this question go here, one per line: 'Test: &lt;what I do&gt; -&gt; &lt;what I should see&gt;'. Skip logic, Mandatory and limits already become tests automatically.</t>
       </text>
     </comment>
   </commentList>
@@ -8344,14 +8328,29 @@
     <author>LIME</author>
   </authors>
   <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Step = form code + step number (F17-1, F17-2...). Action = what I do. Description = what I should see. One scenario = the steps sharing the same prefix.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>LIME</author>
+  </authors>
+  <commentList>
     <comment ref="B8" authorId="0" shapeId="0">
       <text>
-        <t>Filled from scripts/metadata-check.py --all (mandatory, limits, questions present).</t>
+        <t>From scripts/metadata-check.py --all: questions present, mandatory, limits.</t>
       </text>
     </comment>
     <comment ref="D8" authorId="0" shapeId="0">
       <text>
-        <t>Filled from scripts/metadata-check.py --all (every Skip logic rule, both ways).</t>
+        <t>From scripts/metadata-check.py --all: every Skip logic rule, both ways.</t>
       </text>
     </comment>
   </commentList>
@@ -9145,7 +9144,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BR17"/>
+  <dimension ref="A1:BP17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col outlineLevel="1" width="21.42578125" customWidth="1" min="1" max="1"/>
@@ -9191,10 +9190,8 @@
     <col width="48.42578125" customWidth="1" min="62" max="62"/>
     <col width="45" customWidth="1" min="63" max="63"/>
     <col width="18.5703125" customWidth="1" min="64" max="64"/>
-    <col hidden="1" width="13" customWidth="1" min="66" max="67"/>
+    <col hidden="1" min="66" max="67"/>
     <col width="21.42578125" customWidth="1" min="68" max="68"/>
-    <col width="42" customWidth="1" min="69" max="69"/>
-    <col width="42" customWidth="1" min="70" max="70"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.35" customHeight="1">
@@ -9249,11 +9246,6 @@
           <t>F17-Surgery admission form</t>
         </is>
       </c>
-      <c r="BQ1" s="799" t="inlineStr">
-        <is>
-          <t>NEW (optional): only for what the columns above cannot express</t>
-        </is>
-      </c>
     </row>
     <row r="2" ht="30" customFormat="1" customHeight="1" s="1">
       <c r="A2" s="2" t="inlineStr">
@@ -9594,16 +9586,6 @@
       <c r="BP2" s="2" t="inlineStr">
         <is>
           <t>Question ID</t>
-        </is>
-      </c>
-      <c r="BQ2" s="800" t="inlineStr">
-        <is>
-          <t>Test - If I do...</t>
-        </is>
-      </c>
-      <c r="BR2" s="800" t="inlineStr">
-        <is>
-          <t>Test - I should see...</t>
         </is>
       </c>
     </row>
@@ -9725,6 +9707,7 @@
           <t>تاريخ الدخول</t>
         </is>
       </c>
+      <c r="AY3" t="inlineStr"/>
       <c r="AZ3" t="inlineStr">
         <is>
           <t>بيانات القبول</t>
@@ -9898,6 +9881,7 @@
       <c r="BO4" s="41" t="n">
         <v>4</v>
       </c>
+      <c r="BP4" t="inlineStr"/>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -10008,6 +9992,7 @@
       <c r="BO5" s="41" t="n">
         <v>4</v>
       </c>
+      <c r="BP5" t="inlineStr"/>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" t="inlineStr">
@@ -10128,6 +10113,7 @@
           <t>نوع الدخول</t>
         </is>
       </c>
+      <c r="AY6" t="inlineStr"/>
       <c r="AZ6" t="inlineStr">
         <is>
           <t>بيانات القبول</t>
@@ -10309,6 +10295,7 @@
           <t>تمت إحالته إلى منظمة أطباء بلا حدود</t>
         </is>
       </c>
+      <c r="AY7" t="inlineStr"/>
       <c r="AZ7" t="inlineStr">
         <is>
           <t>بيانات القبول</t>
@@ -10494,6 +10481,7 @@
           <t>مُشار إليه - من قبل من / من أين</t>
         </is>
       </c>
+      <c r="AY8" t="inlineStr"/>
       <c r="AZ8" t="inlineStr">
         <is>
           <t>بيانات القبول</t>
@@ -10678,6 +10666,7 @@
           <t>إذا كان غير ذلك، حدد</t>
         </is>
       </c>
+      <c r="AY9" t="inlineStr"/>
       <c r="AZ9" t="inlineStr">
         <is>
           <t>بيانات القبول</t>
@@ -10864,6 +10853,7 @@
           <t>المريض القادم من</t>
         </is>
       </c>
+      <c r="AY10" t="inlineStr"/>
       <c r="AZ10" t="inlineStr">
         <is>
           <t>بيانات القبول</t>
@@ -11048,6 +11038,7 @@
           <t>إذا كان غير ذلك، حدد</t>
         </is>
       </c>
+      <c r="AY11" t="inlineStr"/>
       <c r="AZ11" t="inlineStr">
         <is>
           <t>بيانات القبول</t>
@@ -11220,6 +11211,7 @@
           <t>الوقت منذ ظهور الأعراض/الإصابة حتى الدخول إلى المستشفى (بالساعات)</t>
         </is>
       </c>
+      <c r="AY12" t="inlineStr"/>
       <c r="AZ12" t="inlineStr">
         <is>
           <t>تفاصيل القبول</t>
@@ -11397,6 +11389,7 @@
       <c r="BO13" s="41" t="n">
         <v>4</v>
       </c>
+      <c r="BP13" t="inlineStr"/>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" t="inlineStr">
@@ -11573,7 +11566,11 @@
       </c>
       <c r="BI14" s="665" t="n"/>
       <c r="BJ14" s="665" t="n"/>
-      <c r="BK14" s="32" t="n"/>
+      <c r="BK14" s="799" t="inlineStr">
+        <is>
+          <t>Test: Enter 450 -&gt; A warning: the weight is not plausible</t>
+        </is>
+      </c>
       <c r="BN14" t="inlineStr">
         <is>
           <t>F17-Surgery admission form|9e3c4083-21bd-42d4-a2b5-657bc0b8a4a5</t>
@@ -11585,16 +11582,6 @@
       <c r="BP14" t="inlineStr">
         <is>
           <t>rfe-forms-weightAtAdmission</t>
-        </is>
-      </c>
-      <c r="BQ14" s="801" t="inlineStr">
-        <is>
-          <t>Enter 450</t>
-        </is>
-      </c>
-      <c r="BR14" s="801" t="inlineStr">
-        <is>
-          <t>A warning or refusal: the weight is not plausible</t>
         </is>
       </c>
     </row>
@@ -11706,6 +11693,7 @@
           <t>التعليقات</t>
         </is>
       </c>
+      <c r="AY15" t="inlineStr"/>
       <c r="AZ15" t="inlineStr">
         <is>
           <t>تفاصيل القبول</t>
@@ -11866,6 +11854,7 @@
           <t>وصف الفحوصات والأدوية الجديدة من سلة الطلبات عند الضرورة (بعد إغلاق هذا النموذج)</t>
         </is>
       </c>
+      <c r="AY16" t="inlineStr"/>
       <c r="AZ16" t="inlineStr">
         <is>
           <t>تفاصيل القبول</t>
@@ -12030,6 +12019,7 @@
           <t>طلب الأدوية</t>
         </is>
       </c>
+      <c r="AY17" t="inlineStr"/>
       <c r="AZ17" t="inlineStr">
         <is>
           <t>تفاصيل القبول</t>
@@ -12077,7 +12067,11 @@
       </c>
       <c r="BI17" s="665" t="n"/>
       <c r="BJ17" s="670" t="n"/>
-      <c r="BK17" s="32" t="n"/>
+      <c r="BK17" s="799" t="inlineStr">
+        <is>
+          <t>Test: Click « Order medications » -&gt; The order basket opens for this patient</t>
+        </is>
+      </c>
       <c r="BN17" t="inlineStr">
         <is>
           <t>F17-Surgery admission form|WORKSPACE</t>
@@ -12089,22 +12083,12 @@
       <c r="BP17" s="57" t="inlineStr">
         <is>
           <t>rfe-forms-orderMedications</t>
-        </is>
-      </c>
-      <c r="BQ17" s="801" t="inlineStr">
-        <is>
-          <t>Click « Order medications »</t>
-        </is>
-      </c>
-      <c r="BR17" s="801" t="inlineStr">
-        <is>
-          <t>The order basket opens for this patient</t>
         </is>
       </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <autoFilter ref="A2:BR17"/>
+  <autoFilter ref="A2:BP17"/>
   <mergeCells count="5">
     <mergeCell ref="BA1:BF1"/>
     <mergeCell ref="S1:X1"/>
@@ -12141,170 +12125,160 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr codeName="Sheet24">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="14.45"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="4"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="7"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="802" t="inlineStr">
-        <is>
-          <t>Tests that are not about a single question: patient journeys, several forms, roles and access, reports. One row per test.</t>
+    <row r="1" ht="26.25" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Permission</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Comment</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Form</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Who (role, site)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>If I do...</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>I should see...</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Comments</t>
+      <c r="A2" s="799" t="inlineStr">
+        <is>
+          <t>F17-1</t>
+        </is>
+      </c>
+      <c r="B2" s="799" t="inlineStr">
+        <is>
+          <t>Save a Surgery Admission form for a patient with an active visit</t>
+        </is>
+      </c>
+      <c r="C2" s="799" t="inlineStr">
+        <is>
+          <t>The admission appears in the visit with its admission date</t>
+        </is>
+      </c>
+      <c r="D2" s="799" t="inlineStr">
+        <is>
+          <t>Fictitious patient, active visit</t>
+        </is>
+      </c>
+      <c r="E2" s="799" t="inlineStr">
+        <is>
+          <t>Surgeon, Mosul</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="801" t="inlineStr">
-        <is>
-          <t>F17-Surgery Admission</t>
-        </is>
-      </c>
-      <c r="B3" s="801" t="inlineStr">
+      <c r="A3" s="799" t="inlineStr">
+        <is>
+          <t>F17-2</t>
+        </is>
+      </c>
+      <c r="B3" s="799" t="inlineStr">
+        <is>
+          <t>Open Surgery Discharge (F18) for the same patient</t>
+        </is>
+      </c>
+      <c r="C3" s="799" t="inlineStr">
+        <is>
+          <t>The admission date is shown in the discharge form</t>
+        </is>
+      </c>
+      <c r="E3" s="799" t="inlineStr">
         <is>
           <t>Surgeon, Mosul</t>
-        </is>
-      </c>
-      <c r="C3" s="801" t="inlineStr">
-        <is>
-          <t>Save a Surgery Admission form, then open the patient chart</t>
-        </is>
-      </c>
-      <c r="D3" s="801" t="inlineStr">
-        <is>
-          <t>The admission appears in the visit with its admission date</t>
-        </is>
-      </c>
-      <c r="E3" s="801" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F3" s="801" t="inlineStr">
-        <is>
-          <t>Example</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="801" t="inlineStr">
-        <is>
-          <t>F35-MH-PHQ-9</t>
-        </is>
-      </c>
-      <c r="B4" s="801" t="inlineStr">
+      <c r="A4" s="799" t="inlineStr">
+        <is>
+          <t>F35-1</t>
+        </is>
+      </c>
+      <c r="B4" s="799" t="inlineStr">
+        <is>
+          <t>Answer « Nearly every day (3 points) » to the 9 PHQ-9 questions</t>
+        </is>
+      </c>
+      <c r="C4" s="799" t="inlineStr">
+        <is>
+          <t>PHQ-9 score = 27</t>
+        </is>
+      </c>
+      <c r="E4" s="799" t="inlineStr">
         <is>
           <t>Mental health clinician, all sites</t>
-        </is>
-      </c>
-      <c r="C4" s="801" t="inlineStr">
-        <is>
-          <t>Answer « Nearly every day (3 points) » to the 9 questions</t>
-        </is>
-      </c>
-      <c r="D4" s="801" t="inlineStr">
-        <is>
-          <t>PHQ-9 score = 27</t>
-        </is>
-      </c>
-      <c r="E4" s="801" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F4" s="801" t="inlineStr">
-        <is>
-          <t>Example</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="801" t="inlineStr">
-        <is>
-          <t>(Roles)</t>
-        </is>
-      </c>
-      <c r="B5" s="801" t="inlineStr">
-        <is>
-          <t>Matsapha, « Clinical » role</t>
-        </is>
-      </c>
-      <c r="C5" s="801" t="inlineStr">
+      <c r="A5" s="799" t="inlineStr">
+        <is>
+          <t>ROLES-1</t>
+        </is>
+      </c>
+      <c r="B5" s="799" t="inlineStr">
         <is>
           <t>Open a patient chart</t>
         </is>
       </c>
-      <c r="D5" s="801" t="inlineStr">
+      <c r="C5" s="799" t="inlineStr">
         <is>
           <t>No « Delete » button for visits or encounters</t>
         </is>
       </c>
-      <c r="E5" s="801" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="F5" s="801" t="inlineStr">
-        <is>
-          <t>Example</t>
+      <c r="E5" s="799" t="inlineStr">
+        <is>
+          <t>Matsapha « Clinical » role</t>
+        </is>
+      </c>
+      <c r="F5" s="799" t="inlineStr">
+        <is>
+          <t>No Delete privileges</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:G500"/>
-  <dataValidations count="1">
-    <dataValidation sqref="E3:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Critical,Normal"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -12597,26 +12571,21 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="803" t="inlineStr">
+      <c r="A8" s="799" t="inlineStr">
         <is>
           <t>F17-Surgery Admission</t>
         </is>
       </c>
-      <c r="B8" s="803" t="inlineStr">
+      <c r="B8" s="799" t="inlineStr">
         <is>
           <t>Auto, Oct 13: ✅ 2/2</t>
         </is>
       </c>
-      <c r="C8" s="803" t="n"/>
-      <c r="D8" s="803" t="inlineStr">
+      <c r="D8" s="799" t="inlineStr">
         <is>
           <t>Auto, Oct 13: ✅ 8/8</t>
         </is>
       </c>
-      <c r="E8" s="803" t="n"/>
-      <c r="F8" s="803" t="n"/>
-      <c r="G8" s="803" t="n"/>
-      <c r="H8" s="803" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12978,25 +12947,24 @@
       <c r="D28" s="238" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="802" t="inlineStr">
+      <c r="A30" s="800" t="inlineStr">
         <is>
           <t>Tests</t>
         </is>
       </c>
-      <c r="B30" s="612" t="inlineStr">
-        <is>
-          <t>Skip logic, Mandatory and Lower/Upper limit are turned into tests automatically. Use the 'Test - If I do...' / 'Test - I should see...' columns only for other rules of a question (calculations, plausibility, buttons), and the 'Test Scenarios' tab for tests across questions or forms. Write the expected result precisely ('score = 27', not 'works').</t>
-        </is>
-      </c>
-      <c r="C30" s="612" t="inlineStr">
-        <is>
-          <t>If I do: Enter 450 in 'Weight at admission (in kg)'
-I should see: a warning, the weight is not plausible</t>
-        </is>
-      </c>
-      <c r="D30" s="612" t="inlineStr">
-        <is>
-          <t>I should see: it works</t>
+      <c r="B30" s="799" t="inlineStr">
+        <is>
+          <t>Skip logic, Mandatory and Lower/Upper limit become tests automatically. Other tests on a question: in 'Comments', one per line, 'Test: &lt;what I do&gt; -&gt; &lt;what I should see&gt;'. Tests across questions or forms: 'User flow template' tab (Action = what I do, Description = what I should see).</t>
+        </is>
+      </c>
+      <c r="C30" s="799" t="inlineStr">
+        <is>
+          <t>Test: Enter 450 -&gt; A warning: the weight is not plausible</t>
+        </is>
+      </c>
+      <c r="D30" s="799" t="inlineStr">
+        <is>
+          <t>Test: weight works</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
(docs) Add non-form examples to the metadata test template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U6uYJ2YYNCsnP72DpH3o5o
</commit_message>
<xml_diff>
--- a/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
+++ b/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
@@ -9190,7 +9190,7 @@
     <col width="48.42578125" customWidth="1" min="62" max="62"/>
     <col width="45" customWidth="1" min="63" max="63"/>
     <col width="18.5703125" customWidth="1" min="64" max="64"/>
-    <col hidden="1" min="66" max="67"/>
+    <col hidden="1" width="13" customWidth="1" min="66" max="67"/>
     <col width="21.42578125" customWidth="1" min="68" max="68"/>
   </cols>
   <sheetData>
@@ -9707,7 +9707,6 @@
           <t>تاريخ الدخول</t>
         </is>
       </c>
-      <c r="AY3" t="inlineStr"/>
       <c r="AZ3" t="inlineStr">
         <is>
           <t>بيانات القبول</t>
@@ -9881,7 +9880,6 @@
       <c r="BO4" s="41" t="n">
         <v>4</v>
       </c>
-      <c r="BP4" t="inlineStr"/>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -9992,7 +9990,6 @@
       <c r="BO5" s="41" t="n">
         <v>4</v>
       </c>
-      <c r="BP5" t="inlineStr"/>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" t="inlineStr">
@@ -10113,7 +10110,6 @@
           <t>نوع الدخول</t>
         </is>
       </c>
-      <c r="AY6" t="inlineStr"/>
       <c r="AZ6" t="inlineStr">
         <is>
           <t>بيانات القبول</t>
@@ -10295,7 +10291,6 @@
           <t>تمت إحالته إلى منظمة أطباء بلا حدود</t>
         </is>
       </c>
-      <c r="AY7" t="inlineStr"/>
       <c r="AZ7" t="inlineStr">
         <is>
           <t>بيانات القبول</t>
@@ -10481,7 +10476,6 @@
           <t>مُشار إليه - من قبل من / من أين</t>
         </is>
       </c>
-      <c r="AY8" t="inlineStr"/>
       <c r="AZ8" t="inlineStr">
         <is>
           <t>بيانات القبول</t>
@@ -10666,7 +10660,6 @@
           <t>إذا كان غير ذلك، حدد</t>
         </is>
       </c>
-      <c r="AY9" t="inlineStr"/>
       <c r="AZ9" t="inlineStr">
         <is>
           <t>بيانات القبول</t>
@@ -10853,7 +10846,6 @@
           <t>المريض القادم من</t>
         </is>
       </c>
-      <c r="AY10" t="inlineStr"/>
       <c r="AZ10" t="inlineStr">
         <is>
           <t>بيانات القبول</t>
@@ -11038,7 +11030,6 @@
           <t>إذا كان غير ذلك، حدد</t>
         </is>
       </c>
-      <c r="AY11" t="inlineStr"/>
       <c r="AZ11" t="inlineStr">
         <is>
           <t>بيانات القبول</t>
@@ -11211,7 +11202,6 @@
           <t>الوقت منذ ظهور الأعراض/الإصابة حتى الدخول إلى المستشفى (بالساعات)</t>
         </is>
       </c>
-      <c r="AY12" t="inlineStr"/>
       <c r="AZ12" t="inlineStr">
         <is>
           <t>تفاصيل القبول</t>
@@ -11389,7 +11379,6 @@
       <c r="BO13" s="41" t="n">
         <v>4</v>
       </c>
-      <c r="BP13" t="inlineStr"/>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" t="inlineStr">
@@ -11693,7 +11682,6 @@
           <t>التعليقات</t>
         </is>
       </c>
-      <c r="AY15" t="inlineStr"/>
       <c r="AZ15" t="inlineStr">
         <is>
           <t>تفاصيل القبول</t>
@@ -11854,7 +11842,6 @@
           <t>وصف الفحوصات والأدوية الجديدة من سلة الطلبات عند الضرورة (بعد إغلاق هذا النموذج)</t>
         </is>
       </c>
-      <c r="AY16" t="inlineStr"/>
       <c r="AZ16" t="inlineStr">
         <is>
           <t>تفاصيل القبول</t>
@@ -12019,7 +12006,6 @@
           <t>طلب الأدوية</t>
         </is>
       </c>
-      <c r="AY17" t="inlineStr"/>
       <c r="AZ17" t="inlineStr">
         <is>
           <t>تفاصيل القبول</t>
@@ -12129,7 +12115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="14.45"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12273,6 +12259,50 @@
       <c r="F5" s="799" t="inlineStr">
         <is>
           <t>No Delete privileges</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="799" t="inlineStr">
+        <is>
+          <t>DHIS2-1</t>
+        </is>
+      </c>
+      <c r="B6" s="799" t="inlineStr">
+        <is>
+          <t>Save an F17 form, wait for the nightly sync</t>
+        </is>
+      </c>
+      <c r="C6" s="799" t="inlineStr">
+        <is>
+          <t>The admission appears in DHIS2 with the right date</t>
+        </is>
+      </c>
+      <c r="E6" s="799" t="inlineStr">
+        <is>
+          <t>Data officer</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="799" t="inlineStr">
+        <is>
+          <t>REPORT-1</t>
+        </is>
+      </c>
+      <c r="B7" s="799" t="inlineStr">
+        <is>
+          <t>Run the monthly mental health report for September</t>
+        </is>
+      </c>
+      <c r="C7" s="799" t="inlineStr">
+        <is>
+          <t>The number of new patients matches the patient list</t>
+        </is>
+      </c>
+      <c r="E7" s="799" t="inlineStr">
+        <is>
+          <t>MH manager</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
(docs) Add role and app examples to the metadata test template
Role examples come from the User roles and privileges matrix; app
examples from the Patient Identifiers, Patient Sticker, Appointment
Service Definitions and Visit Types tabs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U6uYJ2YYNCsnP72DpH3o5o
</commit_message>
<xml_diff>
--- a/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
+++ b/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
@@ -12115,7 +12115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="14.45"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12123,8 +12123,8 @@
     <col width="50" customWidth="1" min="3" max="4"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="7"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="6" max="7"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="26.25" customHeight="1">
@@ -12187,7 +12187,7 @@
       </c>
       <c r="E2" s="799" t="inlineStr">
         <is>
-          <t>Surgeon, Mosul</t>
+          <t>Surgeon</t>
         </is>
       </c>
     </row>
@@ -12209,7 +12209,7 @@
       </c>
       <c r="E3" s="799" t="inlineStr">
         <is>
-          <t>Surgeon, Mosul</t>
+          <t>Surgeon</t>
         </is>
       </c>
     </row>
@@ -12231,7 +12231,7 @@
       </c>
       <c r="E4" s="799" t="inlineStr">
         <is>
-          <t>Mental health clinician, all sites</t>
+          <t>MH psychologist</t>
         </is>
       </c>
     </row>
@@ -12243,64 +12243,273 @@
       </c>
       <c r="B5" s="799" t="inlineStr">
         <is>
-          <t>Open a patient chart</t>
+          <t>Register a new patient, then open their patient file</t>
         </is>
       </c>
       <c r="C5" s="799" t="inlineStr">
         <is>
-          <t>No « Delete » button for visits or encounters</t>
+          <t>Registration works; the patient file (clinical tabs) is not accessible</t>
         </is>
       </c>
       <c r="E5" s="799" t="inlineStr">
         <is>
-          <t>Matsapha « Clinical » role</t>
+          <t>Registration Clerk</t>
         </is>
       </c>
       <c r="F5" s="799" t="inlineStr">
         <is>
-          <t>No Delete privileges</t>
+          <t>Patients &gt; Create: x; See patient file: blank</t>
+        </is>
+      </c>
+      <c r="G5" s="799" t="inlineStr">
+        <is>
+          <t>From the User roles and privileges tab</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="799" t="inlineStr">
         <is>
-          <t>DHIS2-1</t>
+          <t>ROLES-2</t>
         </is>
       </c>
       <c r="B6" s="799" t="inlineStr">
         <is>
-          <t>Save an F17 form, wait for the nightly sync</t>
+          <t>Open a patient file and try to order a lab test</t>
         </is>
       </c>
       <c r="C6" s="799" t="inlineStr">
         <is>
-          <t>The admission appears in DHIS2 with the right date</t>
+          <t>No lab order option</t>
         </is>
       </c>
       <c r="E6" s="799" t="inlineStr">
         <is>
-          <t>Data officer</t>
+          <t>MH counselor</t>
+        </is>
+      </c>
+      <c r="F6" s="799" t="inlineStr">
+        <is>
+          <t>Lab &gt; Order lab test: blank</t>
+        </is>
+      </c>
+      <c r="G6" s="799" t="inlineStr">
+        <is>
+          <t>From the User roles and privileges tab</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="799" t="inlineStr">
         <is>
+          <t>ROLES-3</t>
+        </is>
+      </c>
+      <c r="B7" s="799" t="inlineStr">
+        <is>
+          <t>Open a patient file, go to Vitals</t>
+        </is>
+      </c>
+      <c r="C7" s="799" t="inlineStr">
+        <is>
+          <t>Vitals are visible, no « Add » button</t>
+        </is>
+      </c>
+      <c r="E7" s="799" t="inlineStr">
+        <is>
+          <t>MedCo</t>
+        </is>
+      </c>
+      <c r="F7" s="799" t="inlineStr">
+        <is>
+          <t>Vitals &gt; View: x; Add: blank</t>
+        </is>
+      </c>
+      <c r="G7" s="799" t="inlineStr">
+        <is>
+          <t>From the User roles and privileges tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="799" t="inlineStr">
+        <is>
+          <t>ROLES-4</t>
+        </is>
+      </c>
+      <c r="B8" s="799" t="inlineStr">
+        <is>
+          <t>Open a past visit and try to edit it</t>
+        </is>
+      </c>
+      <c r="C8" s="799" t="inlineStr">
+        <is>
+          <t>Editing is refused</t>
+        </is>
+      </c>
+      <c r="E8" s="799" t="inlineStr">
+        <is>
+          <t>MH psychologist</t>
+        </is>
+      </c>
+      <c r="F8" s="799" t="inlineStr">
+        <is>
+          <t>Visits &gt; Edit: blank</t>
+        </is>
+      </c>
+      <c r="G8" s="799" t="inlineStr">
+        <is>
+          <t>From the User roles and privileges tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="799" t="inlineStr">
+        <is>
+          <t>REG-1</t>
+        </is>
+      </c>
+      <c r="B9" s="799" t="inlineStr">
+        <is>
+          <t>Register a new patient</t>
+        </is>
+      </c>
+      <c r="C9" s="799" t="inlineStr">
+        <is>
+          <t>An MSF ID is generated with the prefix IQ146- and at most 16 characters</t>
+        </is>
+      </c>
+      <c r="E9" s="799" t="inlineStr">
+        <is>
+          <t>Registration Clerk</t>
+        </is>
+      </c>
+      <c r="G9" s="799" t="inlineStr">
+        <is>
+          <t>From the Patient Identifiers tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="799" t="inlineStr">
+        <is>
+          <t>PRINT-1</t>
+        </is>
+      </c>
+      <c r="B10" s="799" t="inlineStr">
+        <is>
+          <t>Print the patient sticker</t>
+        </is>
+      </c>
+      <c r="C10" s="799" t="inlineStr">
+        <is>
+          <t>Shows Patient ID, first and last name, gender and date of birth, in Arabic</t>
+        </is>
+      </c>
+      <c r="E10" s="799" t="inlineStr">
+        <is>
+          <t>Registration Clerk</t>
+        </is>
+      </c>
+      <c r="G10" s="799" t="inlineStr">
+        <is>
+          <t>From the Patient Sticker tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="799" t="inlineStr">
+        <is>
+          <t>APPT-1</t>
+        </is>
+      </c>
+      <c r="B11" s="799" t="inlineStr">
+        <is>
+          <t>Book an appointment for a patient</t>
+        </is>
+      </c>
+      <c r="C11" s="799" t="inlineStr">
+        <is>
+          <t>Services offered: General Medicine, Outpatient Department, Rehabilitation, Mental Health</t>
+        </is>
+      </c>
+      <c r="E11" s="799" t="inlineStr">
+        <is>
+          <t>MH psychologist</t>
+        </is>
+      </c>
+      <c r="G11" s="799" t="inlineStr">
+        <is>
+          <t>From the Appointment Service Definitions tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="799" t="inlineStr">
+        <is>
+          <t>VISIT-1</t>
+        </is>
+      </c>
+      <c r="B12" s="799" t="inlineStr">
+        <is>
+          <t>Start a visit</t>
+        </is>
+      </c>
+      <c r="C12" s="799" t="inlineStr">
+        <is>
+          <t>Visit types offered: Facility Visit, Home Visit, OPD Visit, Offline Visit, Group Session</t>
+        </is>
+      </c>
+      <c r="E12" s="799" t="inlineStr">
+        <is>
+          <t>MH psychologist</t>
+        </is>
+      </c>
+      <c r="G12" s="799" t="inlineStr">
+        <is>
+          <t>From the Visit Types tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="799" t="inlineStr">
+        <is>
+          <t>DHIS2-1</t>
+        </is>
+      </c>
+      <c r="B13" s="799" t="inlineStr">
+        <is>
+          <t>Save an F17 form, wait for the next DHIS2 sync</t>
+        </is>
+      </c>
+      <c r="C13" s="799" t="inlineStr">
+        <is>
+          <t>The admission appears in DHIS2 with the right date</t>
+        </is>
+      </c>
+      <c r="E13" s="799" t="inlineStr">
+        <is>
+          <t>Data officer</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="799" t="inlineStr">
+        <is>
           <t>REPORT-1</t>
         </is>
       </c>
-      <c r="B7" s="799" t="inlineStr">
-        <is>
-          <t>Run the monthly mental health report for September</t>
-        </is>
-      </c>
-      <c r="C7" s="799" t="inlineStr">
+      <c r="B14" s="799" t="inlineStr">
+        <is>
+          <t>Run the monthly mental health report for last month</t>
+        </is>
+      </c>
+      <c r="C14" s="799" t="inlineStr">
         <is>
           <t>The number of new patients matches the patient list</t>
         </is>
       </c>
-      <c r="E7" s="799" t="inlineStr">
+      <c r="E14" s="799" t="inlineStr">
         <is>
           <t>MH manager</t>
         </is>

</xml_diff>

<commit_message>
(docs) Fix visit type and appointment examples to match the Mosul configuration
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U6uYJ2YYNCsnP72DpH3o5o
</commit_message>
<xml_diff>
--- a/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
+++ b/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
@@ -12430,7 +12430,7 @@
       </c>
       <c r="C11" s="799" t="inlineStr">
         <is>
-          <t>Services offered: General Medicine, Outpatient Department, Rehabilitation, Mental Health</t>
+          <t>Services offered: Mental Health, and the Mental Health sub-services (AB, DT, KA, SA, SK)</t>
         </is>
       </c>
       <c r="E11" s="799" t="inlineStr">
@@ -12440,7 +12440,7 @@
       </c>
       <c r="G11" s="799" t="inlineStr">
         <is>
-          <t>From the Appointment Service Definitions tab</t>
+          <t>Appointment Service Definitions tab is out of date (lists General Medicine, OPD, Rehabilitation): update it first</t>
         </is>
       </c>
     </row>
@@ -12457,7 +12457,7 @@
       </c>
       <c r="C12" s="799" t="inlineStr">
         <is>
-          <t>Visit types offered: Facility Visit, Home Visit, OPD Visit, Offline Visit, Group Session</t>
+          <t>Visit types offered: OPD Visit, ER Visit, IPD Visit, Telehealth</t>
         </is>
       </c>
       <c r="E12" s="799" t="inlineStr">
@@ -12467,7 +12467,7 @@
       </c>
       <c r="G12" s="799" t="inlineStr">
         <is>
-          <t>From the Visit Types tab</t>
+          <t>Visit Types tab is out of date (lists Facility, Home, Offline, Group Session visits): update it first</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
(docs) Ground the test case examples in the Mosul OpenMRS 3 configuration
- Use EMR role names (workbook name in brackets) instead of workbook-only
  roles; drop MedCo, which has no EMR role
- Show two real differences between the privileges matrix and the EMR:
  Clinical diagnosis is no longer locked by "Edit sensitive mental health
  fields" in F31 (it was in F03), and Mental Health Counselor can add
  orders while the matrix says no lab orders
- Use Mosul mental health cases (F31, PHQ-9, per-counselor appointment
  services, DHIS2 sync of F35) and OpenMRS 3 terms
- Reword the weight example: OpenMRS 3 forms refuse out-of-range values,
  they do not show soft warnings
- Align the workbook template's examples with the document

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U6uYJ2YYNCsnP72DpH3o5o
</commit_message>
<xml_diff>
--- a/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
+++ b/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
@@ -11557,7 +11557,7 @@
       <c r="BJ14" s="665" t="n"/>
       <c r="BK14" s="799" t="inlineStr">
         <is>
-          <t>Test: Enter 450 -&gt; A warning: the weight is not plausible</t>
+          <t>Test: Enter 450 -&gt; The value is refused (needs an Upper limit)</t>
         </is>
       </c>
       <c r="BN14" t="inlineStr">
@@ -12167,17 +12167,17 @@
     <row r="2">
       <c r="A2" s="799" t="inlineStr">
         <is>
-          <t>F17-1</t>
+          <t>F31-1</t>
         </is>
       </c>
       <c r="B2" s="799" t="inlineStr">
         <is>
-          <t>Save a Surgery Admission form for a patient with an active visit</t>
+          <t>Save an F31 mhGAP Baseline during an active visit, then open the patient chart</t>
         </is>
       </c>
       <c r="C2" s="799" t="inlineStr">
         <is>
-          <t>The admission appears in the visit with its admission date</t>
+          <t>The form appears under the visit in the Visits tab and in Forms &amp; Notes</t>
         </is>
       </c>
       <c r="D2" s="799" t="inlineStr">
@@ -12187,95 +12187,105 @@
       </c>
       <c r="E2" s="799" t="inlineStr">
         <is>
-          <t>Surgeon</t>
+          <t>Mental Health Counselor (MH counselor)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="799" t="inlineStr">
         <is>
-          <t>F17-2</t>
+          <t>F35-1</t>
         </is>
       </c>
       <c r="B3" s="799" t="inlineStr">
         <is>
-          <t>Open Surgery Discharge (F18) for the same patient</t>
+          <t>Answer « Nearly every day (3 points) » to the 9 PHQ-9 questions</t>
         </is>
       </c>
       <c r="C3" s="799" t="inlineStr">
         <is>
-          <t>The admission date is shown in the discharge form</t>
+          <t>PHQ-9 score = 27</t>
         </is>
       </c>
       <c r="E3" s="799" t="inlineStr">
         <is>
-          <t>Surgeon</t>
+          <t>Mental Health Counselor (MH counselor)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="799" t="inlineStr">
         <is>
-          <t>F35-1</t>
+          <t>ROLES-1</t>
         </is>
       </c>
       <c r="B4" s="799" t="inlineStr">
         <is>
-          <t>Answer « Nearly every day (3 points) » to the 9 PHQ-9 questions</t>
+          <t>Open the patient chart of a mental health patient</t>
         </is>
       </c>
       <c r="C4" s="799" t="inlineStr">
         <is>
-          <t>PHQ-9 score = 27</t>
+          <t>Mental health forms are not visible</t>
         </is>
       </c>
       <c r="E4" s="799" t="inlineStr">
         <is>
-          <t>MH psychologist</t>
+          <t>Registration Officer (Registration Clerk)</t>
+        </is>
+      </c>
+      <c r="F4" s="799" t="inlineStr">
+        <is>
+          <t>No « View Mental Health »</t>
+        </is>
+      </c>
+      <c r="G4" s="799" t="inlineStr">
+        <is>
+          <t>Today: config matches</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="799" t="inlineStr">
         <is>
-          <t>ROLES-1</t>
+          <t>ROLES-2</t>
         </is>
       </c>
       <c r="B5" s="799" t="inlineStr">
         <is>
-          <t>Register a new patient, then open their patient file</t>
+          <t>Open an F31 mhGAP Baseline, go to Clinical diagnosis</t>
         </is>
       </c>
       <c r="C5" s="799" t="inlineStr">
         <is>
-          <t>Registration works; the patient file (clinical tabs) is not accessible</t>
+          <t>The section is read-only</t>
         </is>
       </c>
       <c r="E5" s="799" t="inlineStr">
         <is>
-          <t>Registration Clerk</t>
+          <t>Mental Health Nurse</t>
         </is>
       </c>
       <c r="F5" s="799" t="inlineStr">
         <is>
-          <t>Patients &gt; Create: x; See patient file: blank</t>
+          <t>No « Edit sensitive mental health fields »</t>
         </is>
       </c>
       <c r="G5" s="799" t="inlineStr">
         <is>
-          <t>From the User roles and privileges tab</t>
+          <t>Today: difference, not locked in F31 (was in F03)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="799" t="inlineStr">
         <is>
-          <t>ROLES-2</t>
+          <t>ROLES-3</t>
         </is>
       </c>
       <c r="B6" s="799" t="inlineStr">
         <is>
-          <t>Open a patient file and try to order a lab test</t>
+          <t>Open the order basket, try to order a lab test</t>
         </is>
       </c>
       <c r="C6" s="799" t="inlineStr">
@@ -12285,235 +12295,147 @@
       </c>
       <c r="E6" s="799" t="inlineStr">
         <is>
-          <t>MH counselor</t>
+          <t>Mental Health Counselor (MH counselor)</t>
         </is>
       </c>
       <c r="F6" s="799" t="inlineStr">
         <is>
-          <t>Lab &gt; Order lab test: blank</t>
+          <t>Matrix: Order lab test blank</t>
         </is>
       </c>
       <c r="G6" s="799" t="inlineStr">
         <is>
-          <t>From the User roles and privileges tab</t>
+          <t>Today: difference, the EMR role can add orders</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="799" t="inlineStr">
         <is>
-          <t>ROLES-3</t>
+          <t>APPT-1</t>
         </is>
       </c>
       <c r="B7" s="799" t="inlineStr">
         <is>
-          <t>Open a patient file, go to Vitals</t>
+          <t>Book a follow-up appointment</t>
         </is>
       </c>
       <c r="C7" s="799" t="inlineStr">
         <is>
-          <t>Vitals are visible, no « Add » button</t>
+          <t>One service per counselor: Mental Health - AB, DT, KA, SA, SK</t>
         </is>
       </c>
       <c r="E7" s="799" t="inlineStr">
         <is>
-          <t>MedCo</t>
-        </is>
-      </c>
-      <c r="F7" s="799" t="inlineStr">
-        <is>
-          <t>Vitals &gt; View: x; Add: blank</t>
-        </is>
-      </c>
-      <c r="G7" s="799" t="inlineStr">
-        <is>
-          <t>From the User roles and privileges tab</t>
-        </is>
-      </c>
+          <t>Registration Officer</t>
+        </is>
+      </c>
+      <c r="F7" s="799" t="n"/>
+      <c r="G7" s="799" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="799" t="inlineStr">
         <is>
-          <t>ROLES-4</t>
+          <t>REG-1</t>
         </is>
       </c>
       <c r="B8" s="799" t="inlineStr">
         <is>
-          <t>Open a past visit and try to edit it</t>
+          <t>Register a new patient</t>
         </is>
       </c>
       <c r="C8" s="799" t="inlineStr">
         <is>
-          <t>Editing is refused</t>
+          <t>An MSF ID is generated automatically: prefix IQ146-, at most 16 characters</t>
         </is>
       </c>
       <c r="E8" s="799" t="inlineStr">
         <is>
-          <t>MH psychologist</t>
-        </is>
-      </c>
-      <c r="F8" s="799" t="inlineStr">
-        <is>
-          <t>Visits &gt; Edit: blank</t>
-        </is>
-      </c>
+          <t>Registration Officer</t>
+        </is>
+      </c>
+      <c r="F8" s="799" t="n"/>
       <c r="G8" s="799" t="inlineStr">
         <is>
-          <t>From the User roles and privileges tab</t>
+          <t>Today: config matches</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="799" t="inlineStr">
         <is>
-          <t>REG-1</t>
+          <t>VISIT-1</t>
         </is>
       </c>
       <c r="B9" s="799" t="inlineStr">
         <is>
-          <t>Register a new patient</t>
+          <t>Start a visit</t>
         </is>
       </c>
       <c r="C9" s="799" t="inlineStr">
         <is>
-          <t>An MSF ID is generated with the prefix IQ146- and at most 16 characters</t>
+          <t>Visit types offered: OPD Visit, ER Visit, IPD Visit, Telehealth</t>
         </is>
       </c>
       <c r="E9" s="799" t="inlineStr">
         <is>
-          <t>Registration Clerk</t>
+          <t>Mental Health Counselor</t>
         </is>
       </c>
       <c r="G9" s="799" t="inlineStr">
         <is>
-          <t>From the Patient Identifiers tab</t>
+          <t>Visit Types tab is out of date: update it first</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="799" t="inlineStr">
         <is>
-          <t>PRINT-1</t>
+          <t>DHIS2-1</t>
         </is>
       </c>
       <c r="B10" s="799" t="inlineStr">
         <is>
-          <t>Print the patient sticker</t>
+          <t>Save an F35 PHQ-9, wait for the daily DHIS2 sync</t>
         </is>
       </c>
       <c r="C10" s="799" t="inlineStr">
         <is>
-          <t>Shows Patient ID, first and last name, gender and date of birth, in Arabic</t>
+          <t>The PHQ-9 score appears in DHIS2 for that patient</t>
         </is>
       </c>
       <c r="E10" s="799" t="inlineStr">
         <is>
-          <t>Registration Clerk</t>
-        </is>
-      </c>
-      <c r="G10" s="799" t="inlineStr">
-        <is>
-          <t>From the Patient Sticker tab</t>
-        </is>
-      </c>
+          <t>Automatic (daily sync)</t>
+        </is>
+      </c>
+      <c r="G10" s="799" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="799" t="inlineStr">
-        <is>
-          <t>APPT-1</t>
-        </is>
-      </c>
-      <c r="B11" s="799" t="inlineStr">
-        <is>
-          <t>Book an appointment for a patient</t>
-        </is>
-      </c>
-      <c r="C11" s="799" t="inlineStr">
-        <is>
-          <t>Services offered: Mental Health, and the Mental Health sub-services (AB, DT, KA, SA, SK)</t>
-        </is>
-      </c>
-      <c r="E11" s="799" t="inlineStr">
-        <is>
-          <t>MH psychologist</t>
-        </is>
-      </c>
-      <c r="G11" s="799" t="inlineStr">
-        <is>
-          <t>Appointment Service Definitions tab is out of date (lists General Medicine, OPD, Rehabilitation): update it first</t>
-        </is>
-      </c>
+      <c r="A11" s="799" t="n"/>
+      <c r="B11" s="799" t="n"/>
+      <c r="C11" s="799" t="n"/>
+      <c r="E11" s="799" t="n"/>
+      <c r="G11" s="799" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="799" t="inlineStr">
-        <is>
-          <t>VISIT-1</t>
-        </is>
-      </c>
-      <c r="B12" s="799" t="inlineStr">
-        <is>
-          <t>Start a visit</t>
-        </is>
-      </c>
-      <c r="C12" s="799" t="inlineStr">
-        <is>
-          <t>Visit types offered: OPD Visit, ER Visit, IPD Visit, Telehealth</t>
-        </is>
-      </c>
-      <c r="E12" s="799" t="inlineStr">
-        <is>
-          <t>MH psychologist</t>
-        </is>
-      </c>
-      <c r="G12" s="799" t="inlineStr">
-        <is>
-          <t>Visit Types tab is out of date (lists Facility, Home, Offline, Group Session visits): update it first</t>
-        </is>
-      </c>
+      <c r="A12" s="799" t="n"/>
+      <c r="B12" s="799" t="n"/>
+      <c r="C12" s="799" t="n"/>
+      <c r="E12" s="799" t="n"/>
+      <c r="G12" s="799" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="799" t="inlineStr">
-        <is>
-          <t>DHIS2-1</t>
-        </is>
-      </c>
-      <c r="B13" s="799" t="inlineStr">
-        <is>
-          <t>Save an F17 form, wait for the next DHIS2 sync</t>
-        </is>
-      </c>
-      <c r="C13" s="799" t="inlineStr">
-        <is>
-          <t>The admission appears in DHIS2 with the right date</t>
-        </is>
-      </c>
-      <c r="E13" s="799" t="inlineStr">
-        <is>
-          <t>Data officer</t>
-        </is>
-      </c>
+      <c r="A13" s="799" t="n"/>
+      <c r="B13" s="799" t="n"/>
+      <c r="C13" s="799" t="n"/>
+      <c r="E13" s="799" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="799" t="inlineStr">
-        <is>
-          <t>REPORT-1</t>
-        </is>
-      </c>
-      <c r="B14" s="799" t="inlineStr">
-        <is>
-          <t>Run the monthly mental health report for last month</t>
-        </is>
-      </c>
-      <c r="C14" s="799" t="inlineStr">
-        <is>
-          <t>The number of new patients matches the patient list</t>
-        </is>
-      </c>
-      <c r="E14" s="799" t="inlineStr">
-        <is>
-          <t>MH manager</t>
-        </is>
-      </c>
+      <c r="A14" s="799" t="n"/>
+      <c r="B14" s="799" t="n"/>
+      <c r="C14" s="799" t="n"/>
+      <c r="E14" s="799" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13185,6 +13107,7 @@
       <c r="C28" s="238" t="n"/>
       <c r="D28" s="238" t="n"/>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="800" t="inlineStr">
         <is>
@@ -13198,7 +13121,7 @@
       </c>
       <c r="C30" s="799" t="inlineStr">
         <is>
-          <t>Test: Enter 450 -&gt; A warning: the weight is not plausible</t>
+          <t>Test: Enter 450 -&gt; The value is refused (needs an Upper limit)</t>
         </is>
       </c>
       <c r="D30" s="799" t="inlineStr">

</xml_diff>

<commit_message>
(docs) Align the workbook template with the verified examples
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U6uYJ2YYNCsnP72DpH3o5o
</commit_message>
<xml_diff>
--- a/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
+++ b/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
@@ -8307,56 +8307,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>LIME</author>
-  </authors>
-  <commentList>
-    <comment ref="BK2" authorId="0" shapeId="0">
-      <text>
-        <t>Tests on this question go here, one per line: 'Test: &lt;what I do&gt; -&gt; &lt;what I should see&gt;'. Skip logic, Mandatory and limits already become tests automatically.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>LIME</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Step = form code + step number (F17-1, F17-2...). Action = what I do. Description = what I should see. One scenario = the steps sharing the same prefix.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>LIME</author>
-  </authors>
-  <commentList>
-    <comment ref="B8" authorId="0" shapeId="0">
-      <text>
-        <t>From scripts/metadata-check.py --all: questions present, mandatory, limits.</t>
-      </text>
-    </comment>
-    <comment ref="D8" authorId="0" shapeId="0">
-      <text>
-        <t>From scripts/metadata-check.py --all: every Skip logic rule, both ways.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
@@ -11555,11 +11505,7 @@
       </c>
       <c r="BI14" s="665" t="n"/>
       <c r="BJ14" s="665" t="n"/>
-      <c r="BK14" s="799" t="inlineStr">
-        <is>
-          <t>Test: Enter 450 -&gt; The value is refused (needs an Upper limit)</t>
-        </is>
-      </c>
+      <c r="BK14" s="799" t="n"/>
       <c r="BN14" t="inlineStr">
         <is>
           <t>F17-Surgery admission form|9e3c4083-21bd-42d4-a2b5-657bc0b8a4a5</t>
@@ -12055,7 +12001,7 @@
       <c r="BJ17" s="670" t="n"/>
       <c r="BK17" s="799" t="inlineStr">
         <is>
-          <t>Test: Click « Order medications » -&gt; The order basket opens for this patient</t>
+          <t>Test: Click « Order medications » -&gt; The order basket opens</t>
         </is>
       </c>
       <c r="BN17" t="inlineStr">
@@ -12105,7 +12051,6 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -12167,248 +12112,164 @@
     <row r="2">
       <c r="A2" s="799" t="inlineStr">
         <is>
-          <t>F31-1</t>
+          <t>ROLES-1</t>
         </is>
       </c>
       <c r="B2" s="799" t="inlineStr">
         <is>
-          <t>Save an F31 mhGAP Baseline during an active visit, then open the patient chart</t>
+          <t>Open the patient chart of a mental health patient</t>
         </is>
       </c>
       <c r="C2" s="799" t="inlineStr">
         <is>
-          <t>The form appears under the visit in the Visits tab and in Forms &amp; Notes</t>
-        </is>
-      </c>
-      <c r="D2" s="799" t="inlineStr">
-        <is>
-          <t>Fictitious patient, active visit</t>
-        </is>
-      </c>
+          <t>Mental health encounters are not visible</t>
+        </is>
+      </c>
+      <c r="D2" s="799" t="n"/>
       <c r="E2" s="799" t="inlineStr">
         <is>
-          <t>Mental Health Counselor (MH counselor)</t>
+          <t>Registration Officer (Registration Clerk)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="799" t="inlineStr">
         <is>
-          <t>F35-1</t>
+          <t>ROLES-2</t>
         </is>
       </c>
       <c r="B3" s="799" t="inlineStr">
         <is>
-          <t>Answer « Nearly every day (3 points) » to the 9 PHQ-9 questions</t>
+          <t>Open an F31 mhGAP Baseline, go to Clinical diagnosis</t>
         </is>
       </c>
       <c r="C3" s="799" t="inlineStr">
         <is>
-          <t>PHQ-9 score = 27</t>
+          <t>The section is read-only (no « Edit sensitive mental health fields » right)</t>
         </is>
       </c>
       <c r="E3" s="799" t="inlineStr">
         <is>
-          <t>Mental Health Counselor (MH counselor)</t>
+          <t>Mental Health Nurse</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="799" t="inlineStr">
         <is>
-          <t>ROLES-1</t>
+          <t>ROLES-3</t>
         </is>
       </c>
       <c r="B4" s="799" t="inlineStr">
         <is>
-          <t>Open the patient chart of a mental health patient</t>
+          <t>Try to order a lab test</t>
         </is>
       </c>
       <c r="C4" s="799" t="inlineStr">
         <is>
-          <t>Mental health forms are not visible</t>
+          <t>No lab order option (matrix: « Order lab test » blank)</t>
         </is>
       </c>
       <c r="E4" s="799" t="inlineStr">
         <is>
-          <t>Registration Officer (Registration Clerk)</t>
-        </is>
-      </c>
-      <c r="F4" s="799" t="inlineStr">
-        <is>
-          <t>No « View Mental Health »</t>
-        </is>
-      </c>
-      <c r="G4" s="799" t="inlineStr">
-        <is>
-          <t>Today: config matches</t>
-        </is>
-      </c>
+          <t>Mental Health Counselor (MH counselor)</t>
+        </is>
+      </c>
+      <c r="F4" s="799" t="n"/>
+      <c r="G4" s="799" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="799" t="inlineStr">
         <is>
-          <t>ROLES-2</t>
+          <t>APPT-1</t>
         </is>
       </c>
       <c r="B5" s="799" t="inlineStr">
         <is>
-          <t>Open an F31 mhGAP Baseline, go to Clinical diagnosis</t>
+          <t>Book a follow-up appointment</t>
         </is>
       </c>
       <c r="C5" s="799" t="inlineStr">
         <is>
-          <t>The section is read-only</t>
+          <t>Services: Mental Health, and Mental Health - AB, DT, KA, SA, SK</t>
         </is>
       </c>
       <c r="E5" s="799" t="inlineStr">
         <is>
-          <t>Mental Health Nurse</t>
-        </is>
-      </c>
-      <c r="F5" s="799" t="inlineStr">
-        <is>
-          <t>No « Edit sensitive mental health fields »</t>
-        </is>
-      </c>
-      <c r="G5" s="799" t="inlineStr">
-        <is>
-          <t>Today: difference, not locked in F31 (was in F03)</t>
-        </is>
-      </c>
+          <t>Mental Health Counselor</t>
+        </is>
+      </c>
+      <c r="F5" s="799" t="n"/>
+      <c r="G5" s="799" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="799" t="inlineStr">
         <is>
-          <t>ROLES-3</t>
+          <t>REG-1</t>
         </is>
       </c>
       <c r="B6" s="799" t="inlineStr">
         <is>
-          <t>Open the order basket, try to order a lab test</t>
+          <t>Register a new patient</t>
         </is>
       </c>
       <c r="C6" s="799" t="inlineStr">
         <is>
-          <t>No lab order option</t>
+          <t>An MSF ID is generated automatically: prefix IQ146-, at most 16 characters</t>
         </is>
       </c>
       <c r="E6" s="799" t="inlineStr">
         <is>
-          <t>Mental Health Counselor (MH counselor)</t>
-        </is>
-      </c>
-      <c r="F6" s="799" t="inlineStr">
-        <is>
-          <t>Matrix: Order lab test blank</t>
-        </is>
-      </c>
-      <c r="G6" s="799" t="inlineStr">
-        <is>
-          <t>Today: difference, the EMR role can add orders</t>
-        </is>
-      </c>
+          <t>Registration Officer</t>
+        </is>
+      </c>
+      <c r="F6" s="799" t="n"/>
+      <c r="G6" s="799" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="799" t="inlineStr">
         <is>
-          <t>APPT-1</t>
+          <t>DHIS2-1</t>
         </is>
       </c>
       <c r="B7" s="799" t="inlineStr">
         <is>
-          <t>Book a follow-up appointment</t>
+          <t>Save an F31 mhGAP Baseline with a PHQ-9 score</t>
         </is>
       </c>
       <c r="C7" s="799" t="inlineStr">
         <is>
-          <t>One service per counselor: Mental Health - AB, DT, KA, SA, SK</t>
+          <t>After the daily sync (17:00), the PHQ-9 score is in DHIS2</t>
         </is>
       </c>
       <c r="E7" s="799" t="inlineStr">
         <is>
-          <t>Registration Officer</t>
+          <t>Automatic</t>
         </is>
       </c>
       <c r="F7" s="799" t="n"/>
       <c r="G7" s="799" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="799" t="inlineStr">
-        <is>
-          <t>REG-1</t>
-        </is>
-      </c>
-      <c r="B8" s="799" t="inlineStr">
-        <is>
-          <t>Register a new patient</t>
-        </is>
-      </c>
-      <c r="C8" s="799" t="inlineStr">
-        <is>
-          <t>An MSF ID is generated automatically: prefix IQ146-, at most 16 characters</t>
-        </is>
-      </c>
-      <c r="E8" s="799" t="inlineStr">
-        <is>
-          <t>Registration Officer</t>
-        </is>
-      </c>
+      <c r="A8" s="799" t="n"/>
+      <c r="B8" s="799" t="n"/>
+      <c r="C8" s="799" t="n"/>
+      <c r="E8" s="799" t="n"/>
       <c r="F8" s="799" t="n"/>
-      <c r="G8" s="799" t="inlineStr">
-        <is>
-          <t>Today: config matches</t>
-        </is>
-      </c>
+      <c r="G8" s="799" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="799" t="inlineStr">
-        <is>
-          <t>VISIT-1</t>
-        </is>
-      </c>
-      <c r="B9" s="799" t="inlineStr">
-        <is>
-          <t>Start a visit</t>
-        </is>
-      </c>
-      <c r="C9" s="799" t="inlineStr">
-        <is>
-          <t>Visit types offered: OPD Visit, ER Visit, IPD Visit, Telehealth</t>
-        </is>
-      </c>
-      <c r="E9" s="799" t="inlineStr">
-        <is>
-          <t>Mental Health Counselor</t>
-        </is>
-      </c>
-      <c r="G9" s="799" t="inlineStr">
-        <is>
-          <t>Visit Types tab is out of date: update it first</t>
-        </is>
-      </c>
+      <c r="A9" s="799" t="n"/>
+      <c r="B9" s="799" t="n"/>
+      <c r="C9" s="799" t="n"/>
+      <c r="E9" s="799" t="n"/>
+      <c r="G9" s="799" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="799" t="inlineStr">
-        <is>
-          <t>DHIS2-1</t>
-        </is>
-      </c>
-      <c r="B10" s="799" t="inlineStr">
-        <is>
-          <t>Save an F35 PHQ-9, wait for the daily DHIS2 sync</t>
-        </is>
-      </c>
-      <c r="C10" s="799" t="inlineStr">
-        <is>
-          <t>The PHQ-9 score appears in DHIS2 for that patient</t>
-        </is>
-      </c>
-      <c r="E10" s="799" t="inlineStr">
-        <is>
-          <t>Automatic (daily sync)</t>
-        </is>
-      </c>
+      <c r="A10" s="799" t="n"/>
+      <c r="B10" s="799" t="n"/>
+      <c r="C10" s="799" t="n"/>
+      <c r="E10" s="799" t="n"/>
       <c r="G10" s="799" t="n"/>
     </row>
     <row r="11">
@@ -12439,7 +12300,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -12750,7 +12610,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -13116,17 +12975,17 @@
       </c>
       <c r="B30" s="799" t="inlineStr">
         <is>
-          <t>Skip logic, Mandatory and Lower/Upper limit become tests automatically. Other tests on a question: in 'Comments', one per line, 'Test: &lt;what I do&gt; -&gt; &lt;what I should see&gt;'. Tests across questions or forms: 'User flow template' tab (Action = what I do, Description = what I should see).</t>
+          <t>Other tests on a question: in 'Comments', 'Test: &lt;what I do&gt; -&gt; &lt;what I should see&gt;'. Tests across questions or forms: 'User flow template' (Action = what I do, Description = what I should see).</t>
         </is>
       </c>
       <c r="C30" s="799" t="inlineStr">
         <is>
-          <t>Test: Enter 450 -&gt; The value is refused (needs an Upper limit)</t>
+          <t>Test: Click « Order medications » -&gt; The order basket opens</t>
         </is>
       </c>
       <c r="D30" s="799" t="inlineStr">
         <is>
-          <t>Test: weight works</t>
+          <t>Test: button works</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
(docs) Make the examples Mosul implementation test cases
Form test cases live with the forms and run once in the distro, so the
document now covers what is specific to the Mosul site, each row taken
from the Mosul configuration: login locations, languages, MSF ID
generator, Iraq address hierarchy, unidentified patients, identifier
sticker, mental health access, per-counselor appointment services,
visit types and auto-close, 24-hour edit window, retrospective data
entry and the DHIS2 sync. Lists two differences found: lab orders for
Mental Health Counselor, and "Home Visit" in the auto-close list.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U6uYJ2YYNCsnP72DpH3o5o
</commit_message>
<xml_diff>
--- a/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
+++ b/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
@@ -12060,7 +12060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="14.45"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12112,67 +12112,67 @@
     <row r="2">
       <c r="A2" s="799" t="inlineStr">
         <is>
-          <t>ROLES-1</t>
+          <t>LOGIN-1</t>
         </is>
       </c>
       <c r="B2" s="799" t="inlineStr">
         <is>
-          <t>Open the patient chart of a mental health patient</t>
+          <t>Log in</t>
         </is>
       </c>
       <c r="C2" s="799" t="inlineStr">
         <is>
-          <t>Mental health encounters are not visible</t>
+          <t>Two locations offered: Mental Health (MH) / الصحة النفسية, and Registration Counter (REG) / تسجيل المستشفى</t>
         </is>
       </c>
       <c r="D2" s="799" t="n"/>
       <c r="E2" s="799" t="inlineStr">
         <is>
-          <t>Registration Officer (Registration Clerk)</t>
+          <t>Any user</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="799" t="inlineStr">
         <is>
-          <t>ROLES-2</t>
+          <t>LANG-1</t>
         </is>
       </c>
       <c r="B3" s="799" t="inlineStr">
         <is>
-          <t>Open an F31 mhGAP Baseline, go to Clinical diagnosis</t>
+          <t>Change the language</t>
         </is>
       </c>
       <c r="C3" s="799" t="inlineStr">
         <is>
-          <t>The section is read-only (no « Edit sensitive mental health fields » right)</t>
+          <t>English and Arabic offered; English by default</t>
         </is>
       </c>
       <c r="E3" s="799" t="inlineStr">
         <is>
-          <t>Mental Health Nurse</t>
+          <t>Any user</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="799" t="inlineStr">
         <is>
-          <t>ROLES-3</t>
+          <t>REG-1</t>
         </is>
       </c>
       <c r="B4" s="799" t="inlineStr">
         <is>
-          <t>Try to order a lab test</t>
+          <t>Register a new patient</t>
         </is>
       </c>
       <c r="C4" s="799" t="inlineStr">
         <is>
-          <t>No lab order option (matrix: « Order lab test » blank)</t>
+          <t>MSF ID generated automatically (prefix IQ146-, at most 16 characters); Legacy MSF ID optional</t>
         </is>
       </c>
       <c r="E4" s="799" t="inlineStr">
         <is>
-          <t>Mental Health Counselor (MH counselor)</t>
+          <t>Registration Officer</t>
         </is>
       </c>
       <c r="F4" s="799" t="n"/>
@@ -12181,22 +12181,22 @@
     <row r="5">
       <c r="A5" s="799" t="inlineStr">
         <is>
-          <t>APPT-1</t>
+          <t>REG-2</t>
         </is>
       </c>
       <c r="B5" s="799" t="inlineStr">
         <is>
-          <t>Book a follow-up appointment</t>
+          <t>Enter the patient address</t>
         </is>
       </c>
       <c r="C5" s="799" t="inlineStr">
         <is>
-          <t>Services: Mental Health, and Mental Health - AB, DT, KA, SA, SK</t>
+          <t>Address picked level by level: Iraq &gt; Ninawa &gt; district (Mosul, Sinjar, Talafar...) &gt; area</t>
         </is>
       </c>
       <c r="E5" s="799" t="inlineStr">
         <is>
-          <t>Mental Health Counselor</t>
+          <t>Registration Officer</t>
         </is>
       </c>
       <c r="F5" s="799" t="n"/>
@@ -12205,17 +12205,17 @@
     <row r="6">
       <c r="A6" s="799" t="inlineStr">
         <is>
-          <t>REG-1</t>
+          <t>REG-3</t>
         </is>
       </c>
       <c r="B6" s="799" t="inlineStr">
         <is>
-          <t>Register a new patient</t>
+          <t>Register a patient whose name is unknown</t>
         </is>
       </c>
       <c r="C6" s="799" t="inlineStr">
         <is>
-          <t>An MSF ID is generated automatically: prefix IQ146-, at most 16 characters</t>
+          <t>Registration is allowed</t>
         </is>
       </c>
       <c r="E6" s="799" t="inlineStr">
@@ -12229,74 +12229,208 @@
     <row r="7">
       <c r="A7" s="799" t="inlineStr">
         <is>
-          <t>DHIS2-1</t>
+          <t>REG-4</t>
         </is>
       </c>
       <c r="B7" s="799" t="inlineStr">
         <is>
-          <t>Save an F31 mhGAP Baseline with a PHQ-9 score</t>
+          <t>Open the patient chart</t>
         </is>
       </c>
       <c r="C7" s="799" t="inlineStr">
         <is>
-          <t>After the daily sync (17:00), the PHQ-9 score is in DHIS2</t>
+          <t>A « Print identifier sticker » button is available</t>
         </is>
       </c>
       <c r="E7" s="799" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Registration Officer</t>
         </is>
       </c>
       <c r="F7" s="799" t="n"/>
       <c r="G7" s="799" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="799" t="n"/>
-      <c r="B8" s="799" t="n"/>
-      <c r="C8" s="799" t="n"/>
-      <c r="E8" s="799" t="n"/>
+      <c r="A8" s="799" t="inlineStr">
+        <is>
+          <t>ROLES-1</t>
+        </is>
+      </c>
+      <c r="B8" s="799" t="inlineStr">
+        <is>
+          <t>Open the patient chart of a mental health patient</t>
+        </is>
+      </c>
+      <c r="C8" s="799" t="inlineStr">
+        <is>
+          <t>Mental health encounters are not visible</t>
+        </is>
+      </c>
+      <c r="E8" s="799" t="inlineStr">
+        <is>
+          <t>Registration Officer</t>
+        </is>
+      </c>
       <c r="F8" s="799" t="n"/>
       <c r="G8" s="799" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="799" t="n"/>
-      <c r="B9" s="799" t="n"/>
-      <c r="C9" s="799" t="n"/>
-      <c r="E9" s="799" t="n"/>
+      <c r="A9" s="799" t="inlineStr">
+        <is>
+          <t>ROLES-2</t>
+        </is>
+      </c>
+      <c r="B9" s="799" t="inlineStr">
+        <is>
+          <t>Try to order a lab test</t>
+        </is>
+      </c>
+      <c r="C9" s="799" t="inlineStr">
+        <is>
+          <t>No lab order option</t>
+        </is>
+      </c>
+      <c r="E9" s="799" t="inlineStr">
+        <is>
+          <t>Mental Health Counselor</t>
+        </is>
+      </c>
       <c r="G9" s="799" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="799" t="n"/>
-      <c r="B10" s="799" t="n"/>
-      <c r="C10" s="799" t="n"/>
-      <c r="E10" s="799" t="n"/>
+      <c r="A10" s="799" t="inlineStr">
+        <is>
+          <t>APPT-1</t>
+        </is>
+      </c>
+      <c r="B10" s="799" t="inlineStr">
+        <is>
+          <t>Book a follow-up appointment</t>
+        </is>
+      </c>
+      <c r="C10" s="799" t="inlineStr">
+        <is>
+          <t>Services: Mental Health, and Mental Health - AB, DT, KA, SA, SK</t>
+        </is>
+      </c>
+      <c r="E10" s="799" t="inlineStr">
+        <is>
+          <t>Mental Health Counselor</t>
+        </is>
+      </c>
       <c r="G10" s="799" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="799" t="n"/>
-      <c r="B11" s="799" t="n"/>
-      <c r="C11" s="799" t="n"/>
-      <c r="E11" s="799" t="n"/>
+      <c r="A11" s="799" t="inlineStr">
+        <is>
+          <t>VISIT-1</t>
+        </is>
+      </c>
+      <c r="B11" s="799" t="inlineStr">
+        <is>
+          <t>Start a visit</t>
+        </is>
+      </c>
+      <c r="C11" s="799" t="inlineStr">
+        <is>
+          <t>Visit types offered: OPD Visit, ER Visit, IPD Visit, Telehealth</t>
+        </is>
+      </c>
+      <c r="E11" s="799" t="inlineStr">
+        <is>
+          <t>Mental Health Counselor</t>
+        </is>
+      </c>
       <c r="G11" s="799" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="799" t="n"/>
-      <c r="B12" s="799" t="n"/>
-      <c r="C12" s="799" t="n"/>
-      <c r="E12" s="799" t="n"/>
+      <c r="A12" s="799" t="inlineStr">
+        <is>
+          <t>VISIT-2</t>
+        </is>
+      </c>
+      <c r="B12" s="799" t="inlineStr">
+        <is>
+          <t>Leave an OPD or Telehealth visit open</t>
+        </is>
+      </c>
+      <c r="C12" s="799" t="inlineStr">
+        <is>
+          <t>The visit is closed automatically</t>
+        </is>
+      </c>
+      <c r="E12" s="799" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
       <c r="G12" s="799" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="799" t="n"/>
-      <c r="B13" s="799" t="n"/>
-      <c r="C13" s="799" t="n"/>
-      <c r="E13" s="799" t="n"/>
+      <c r="A13" s="799" t="inlineStr">
+        <is>
+          <t>EDIT-1</t>
+        </is>
+      </c>
+      <c r="B13" s="799" t="inlineStr">
+        <is>
+          <t>Edit a form saved more than 24 hours ago</t>
+        </is>
+      </c>
+      <c r="C13" s="799" t="inlineStr">
+        <is>
+          <t>The form can no longer be edited</t>
+        </is>
+      </c>
+      <c r="E13" s="799" t="inlineStr">
+        <is>
+          <t>Mental Health Counselor</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="799" t="n"/>
-      <c r="B14" s="799" t="n"/>
-      <c r="C14" s="799" t="n"/>
-      <c r="E14" s="799" t="n"/>
+      <c r="A14" s="799" t="inlineStr">
+        <is>
+          <t>RDE-1</t>
+        </is>
+      </c>
+      <c r="B14" s="799" t="inlineStr">
+        <is>
+          <t>Enter data for a past visit</t>
+        </is>
+      </c>
+      <c r="C14" s="799" t="inlineStr">
+        <is>
+          <t>Retrospective data entry is available</t>
+        </is>
+      </c>
+      <c r="E14" s="799" t="inlineStr">
+        <is>
+          <t>Mental Health Counselor</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="799" t="inlineStr">
+        <is>
+          <t>DHIS2-1</t>
+        </is>
+      </c>
+      <c r="B15" s="799" t="inlineStr">
+        <is>
+          <t>Save an F31 mhGAP Baseline with a PHQ-9 score</t>
+        </is>
+      </c>
+      <c r="C15" s="799" t="inlineStr">
+        <is>
+          <t>After the daily sync (17:00), the PHQ-9 score is in DHIS2</t>
+        </is>
+      </c>
+      <c r="E15" s="799" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12966,7 +13100,6 @@
       <c r="C28" s="238" t="n"/>
       <c r="D28" s="238" t="n"/>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="800" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
(feat) Make the User flow template scale across sites and releases
The template's User flow template tab keeps its original columns and
adds Area, Site, Release, Priority, Result and Tested on, with
dropdowns, colored results, frozen header and filters. Examples are the
Mosul Release 1 implementation tests plus a Matsapha delete-rights
pair from roles_matsapha.csv.

metadata-check.py --scenarios lists these tests with counts by area and
result, filtered by --site (rows for "All sites" always included) and
--release; form reports now show each test's recorded result.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U6uYJ2YYNCsnP72DpH3o5o
</commit_message>
<xml_diff>
--- a/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
+++ b/docs/testing/metadonnees/Template - Tests in metadata workbook.xlsx
@@ -7,12 +7,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F17-Surgery Admission" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User flow template" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User flow template" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form QA Tracker" sheetId="3" state="hidden" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form Guidance" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'F17-Surgery Admission'!$A$2:$BP$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'User flow template'!$A$1:$M$1000</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +26,7 @@
     <numFmt numFmtId="165" formatCode="[$-2000401]0"/>
     <numFmt numFmtId="166" formatCode="[$-2000000]\d\d\-mmm"/>
   </numFmts>
-  <fonts count="129">
+  <fonts count="130">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -882,6 +883,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF2E75B6"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="63">
@@ -2101,7 +2108,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="801">
+  <cellXfs count="803">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3703,6 +3710,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="128" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="129" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3710,7 +3723,7 @@
     <cellStyle name="Normal 2" xfId="2"/>
     <cellStyle name="Normal 4" xfId="3"/>
   </cellStyles>
-  <dxfs count="518">
+  <dxfs count="521">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -8298,6 +8311,27 @@
       <fill>
         <patternFill patternType="solid">
           <bgColor theme="9" tint="0.7999816888943144"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -12056,384 +12090,966 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr codeName="Sheet24">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="14.45"/>
+  <dimension ref="A1:M17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="4"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="7"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26.25" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="801" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="801" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C1" s="801" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="D1" s="801" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E1" s="801" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="F1" s="801" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="G1" s="801" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="H1" s="801" t="inlineStr">
         <is>
           <t>User</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="I1" s="801" t="inlineStr">
         <is>
           <t>Permission</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="J1" s="801" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="K1" s="801" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="L1" s="801" t="inlineStr">
+        <is>
+          <t>Tested on</t>
+        </is>
+      </c>
+      <c r="M1" s="801" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="799" t="inlineStr">
+      <c r="A2" s="802" t="inlineStr">
         <is>
           <t>LOGIN-1</t>
         </is>
       </c>
-      <c r="B2" s="799" t="inlineStr">
+      <c r="B2" s="802" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C2" s="802" t="inlineStr">
+        <is>
+          <t>Mosul</t>
+        </is>
+      </c>
+      <c r="D2" s="802" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
+      <c r="E2" s="802" t="inlineStr">
         <is>
           <t>Log in</t>
         </is>
       </c>
-      <c r="C2" s="799" t="inlineStr">
+      <c r="F2" s="802" t="inlineStr">
         <is>
           <t>Two locations offered: Mental Health (MH) / الصحة النفسية, and Registration Counter (REG) / تسجيل المستشفى</t>
         </is>
       </c>
-      <c r="D2" s="799" t="n"/>
-      <c r="E2" s="799" t="inlineStr">
+      <c r="G2" s="802" t="n"/>
+      <c r="H2" s="802" t="inlineStr">
         <is>
           <t>Any user</t>
         </is>
       </c>
+      <c r="I2" s="802" t="n"/>
+      <c r="J2" s="802" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K2" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L2" s="802" t="n"/>
+      <c r="M2" s="802" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="799" t="inlineStr">
+      <c r="A3" s="802" t="inlineStr">
         <is>
           <t>LANG-1</t>
         </is>
       </c>
-      <c r="B3" s="799" t="inlineStr">
+      <c r="B3" s="802" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="C3" s="802" t="inlineStr">
+        <is>
+          <t>Mosul</t>
+        </is>
+      </c>
+      <c r="D3" s="802" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
+      <c r="E3" s="802" t="inlineStr">
         <is>
           <t>Change the language</t>
         </is>
       </c>
-      <c r="C3" s="799" t="inlineStr">
+      <c r="F3" s="802" t="inlineStr">
         <is>
           <t>English and Arabic offered; English by default</t>
         </is>
       </c>
-      <c r="E3" s="799" t="inlineStr">
+      <c r="G3" s="802" t="n"/>
+      <c r="H3" s="802" t="inlineStr">
         <is>
           <t>Any user</t>
         </is>
       </c>
+      <c r="I3" s="802" t="n"/>
+      <c r="J3" s="802" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="K3" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L3" s="802" t="n"/>
+      <c r="M3" s="802" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="799" t="inlineStr">
+      <c r="A4" s="802" t="inlineStr">
         <is>
           <t>REG-1</t>
         </is>
       </c>
-      <c r="B4" s="799" t="inlineStr">
+      <c r="B4" s="802" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C4" s="802" t="inlineStr">
+        <is>
+          <t>Mosul</t>
+        </is>
+      </c>
+      <c r="D4" s="802" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
+      <c r="E4" s="802" t="inlineStr">
         <is>
           <t>Register a new patient</t>
         </is>
       </c>
-      <c r="C4" s="799" t="inlineStr">
+      <c r="F4" s="802" t="inlineStr">
         <is>
           <t>MSF ID generated automatically (prefix IQ146-, at most 16 characters); Legacy MSF ID optional</t>
         </is>
       </c>
-      <c r="E4" s="799" t="inlineStr">
+      <c r="G4" s="802" t="inlineStr">
+        <is>
+          <t>Fictitious patient</t>
+        </is>
+      </c>
+      <c r="H4" s="802" t="inlineStr">
         <is>
           <t>Registration Officer</t>
         </is>
       </c>
-      <c r="F4" s="799" t="n"/>
-      <c r="G4" s="799" t="n"/>
+      <c r="I4" s="802" t="n"/>
+      <c r="J4" s="802" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K4" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L4" s="802" t="n"/>
+      <c r="M4" s="802" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="799" t="inlineStr">
+      <c r="A5" s="802" t="inlineStr">
         <is>
           <t>REG-2</t>
         </is>
       </c>
-      <c r="B5" s="799" t="inlineStr">
+      <c r="B5" s="802" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C5" s="802" t="inlineStr">
+        <is>
+          <t>Mosul</t>
+        </is>
+      </c>
+      <c r="D5" s="802" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
+      <c r="E5" s="802" t="inlineStr">
         <is>
           <t>Enter the patient address</t>
         </is>
       </c>
-      <c r="C5" s="799" t="inlineStr">
+      <c r="F5" s="802" t="inlineStr">
         <is>
           <t>Address picked level by level: Iraq &gt; Ninawa &gt; district (Mosul, Sinjar, Talafar...) &gt; area</t>
         </is>
       </c>
-      <c r="E5" s="799" t="inlineStr">
+      <c r="G5" s="802" t="n"/>
+      <c r="H5" s="802" t="inlineStr">
         <is>
           <t>Registration Officer</t>
         </is>
       </c>
-      <c r="F5" s="799" t="n"/>
-      <c r="G5" s="799" t="n"/>
+      <c r="I5" s="802" t="n"/>
+      <c r="J5" s="802" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="K5" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L5" s="802" t="n"/>
+      <c r="M5" s="802" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="799" t="inlineStr">
+      <c r="A6" s="802" t="inlineStr">
         <is>
           <t>REG-3</t>
         </is>
       </c>
-      <c r="B6" s="799" t="inlineStr">
+      <c r="B6" s="802" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C6" s="802" t="inlineStr">
+        <is>
+          <t>Mosul</t>
+        </is>
+      </c>
+      <c r="D6" s="802" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
+      <c r="E6" s="802" t="inlineStr">
         <is>
           <t>Register a patient whose name is unknown</t>
         </is>
       </c>
-      <c r="C6" s="799" t="inlineStr">
+      <c r="F6" s="802" t="inlineStr">
         <is>
           <t>Registration is allowed</t>
         </is>
       </c>
-      <c r="E6" s="799" t="inlineStr">
+      <c r="G6" s="802" t="n"/>
+      <c r="H6" s="802" t="inlineStr">
         <is>
           <t>Registration Officer</t>
         </is>
       </c>
-      <c r="F6" s="799" t="n"/>
-      <c r="G6" s="799" t="n"/>
+      <c r="I6" s="802" t="n"/>
+      <c r="J6" s="802" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="K6" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L6" s="802" t="n"/>
+      <c r="M6" s="802" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="799" t="inlineStr">
+      <c r="A7" s="802" t="inlineStr">
         <is>
           <t>REG-4</t>
         </is>
       </c>
-      <c r="B7" s="799" t="inlineStr">
+      <c r="B7" s="802" t="inlineStr">
+        <is>
+          <t>Printing</t>
+        </is>
+      </c>
+      <c r="C7" s="802" t="inlineStr">
+        <is>
+          <t>Mosul</t>
+        </is>
+      </c>
+      <c r="D7" s="802" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
+      <c r="E7" s="802" t="inlineStr">
         <is>
           <t>Open the patient chart</t>
         </is>
       </c>
-      <c r="C7" s="799" t="inlineStr">
+      <c r="F7" s="802" t="inlineStr">
         <is>
           <t>A « Print identifier sticker » button is available</t>
         </is>
       </c>
-      <c r="E7" s="799" t="inlineStr">
+      <c r="G7" s="802" t="n"/>
+      <c r="H7" s="802" t="inlineStr">
         <is>
           <t>Registration Officer</t>
         </is>
       </c>
-      <c r="F7" s="799" t="n"/>
-      <c r="G7" s="799" t="n"/>
+      <c r="I7" s="802" t="n"/>
+      <c r="J7" s="802" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="K7" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L7" s="802" t="n"/>
+      <c r="M7" s="802" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="799" t="inlineStr">
+      <c r="A8" s="802" t="inlineStr">
         <is>
           <t>ROLES-1</t>
         </is>
       </c>
-      <c r="B8" s="799" t="inlineStr">
+      <c r="B8" s="802" t="inlineStr">
+        <is>
+          <t>Access and roles</t>
+        </is>
+      </c>
+      <c r="C8" s="802" t="inlineStr">
+        <is>
+          <t>Mosul</t>
+        </is>
+      </c>
+      <c r="D8" s="802" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
+      <c r="E8" s="802" t="inlineStr">
         <is>
           <t>Open the patient chart of a mental health patient</t>
         </is>
       </c>
-      <c r="C8" s="799" t="inlineStr">
+      <c r="F8" s="802" t="inlineStr">
         <is>
           <t>Mental health encounters are not visible</t>
         </is>
       </c>
-      <c r="E8" s="799" t="inlineStr">
+      <c r="G8" s="802" t="n"/>
+      <c r="H8" s="802" t="inlineStr">
         <is>
           <t>Registration Officer</t>
         </is>
       </c>
-      <c r="F8" s="799" t="n"/>
-      <c r="G8" s="799" t="n"/>
+      <c r="I8" s="802" t="inlineStr">
+        <is>
+          <t>No « View Mental Health »</t>
+        </is>
+      </c>
+      <c r="J8" s="802" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K8" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L8" s="802" t="n"/>
+      <c r="M8" s="802" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="799" t="inlineStr">
+      <c r="A9" s="802" t="inlineStr">
         <is>
           <t>ROLES-2</t>
         </is>
       </c>
-      <c r="B9" s="799" t="inlineStr">
+      <c r="B9" s="802" t="inlineStr">
+        <is>
+          <t>Access and roles</t>
+        </is>
+      </c>
+      <c r="C9" s="802" t="inlineStr">
+        <is>
+          <t>Mosul</t>
+        </is>
+      </c>
+      <c r="D9" s="802" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
+      <c r="E9" s="802" t="inlineStr">
         <is>
           <t>Try to order a lab test</t>
         </is>
       </c>
-      <c r="C9" s="799" t="inlineStr">
+      <c r="F9" s="802" t="inlineStr">
         <is>
           <t>No lab order option</t>
         </is>
       </c>
-      <c r="E9" s="799" t="inlineStr">
+      <c r="G9" s="802" t="n"/>
+      <c r="H9" s="802" t="inlineStr">
         <is>
           <t>Mental Health Counselor</t>
         </is>
       </c>
-      <c r="G9" s="799" t="n"/>
+      <c r="I9" s="802" t="inlineStr">
+        <is>
+          <t>Matrix: « Order lab test » blank</t>
+        </is>
+      </c>
+      <c r="J9" s="802" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="K9" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L9" s="802" t="n"/>
+      <c r="M9" s="802" t="inlineStr">
+        <is>
+          <t>Today the EMR role can add orders</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="799" t="inlineStr">
+      <c r="A10" s="802" t="inlineStr">
         <is>
           <t>APPT-1</t>
         </is>
       </c>
-      <c r="B10" s="799" t="inlineStr">
+      <c r="B10" s="802" t="inlineStr">
+        <is>
+          <t>Appointments</t>
+        </is>
+      </c>
+      <c r="C10" s="802" t="inlineStr">
+        <is>
+          <t>Mosul</t>
+        </is>
+      </c>
+      <c r="D10" s="802" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
+      <c r="E10" s="802" t="inlineStr">
         <is>
           <t>Book a follow-up appointment</t>
         </is>
       </c>
-      <c r="C10" s="799" t="inlineStr">
+      <c r="F10" s="802" t="inlineStr">
         <is>
           <t>Services: Mental Health, and Mental Health - AB, DT, KA, SA, SK</t>
         </is>
       </c>
-      <c r="E10" s="799" t="inlineStr">
+      <c r="G10" s="802" t="n"/>
+      <c r="H10" s="802" t="inlineStr">
         <is>
           <t>Mental Health Counselor</t>
         </is>
       </c>
-      <c r="G10" s="799" t="n"/>
+      <c r="I10" s="802" t="n"/>
+      <c r="J10" s="802" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="K10" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L10" s="802" t="n"/>
+      <c r="M10" s="802" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="799" t="inlineStr">
+      <c r="A11" s="802" t="inlineStr">
         <is>
           <t>VISIT-1</t>
         </is>
       </c>
-      <c r="B11" s="799" t="inlineStr">
+      <c r="B11" s="802" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="C11" s="802" t="inlineStr">
+        <is>
+          <t>Mosul</t>
+        </is>
+      </c>
+      <c r="D11" s="802" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
+      <c r="E11" s="802" t="inlineStr">
         <is>
           <t>Start a visit</t>
         </is>
       </c>
-      <c r="C11" s="799" t="inlineStr">
+      <c r="F11" s="802" t="inlineStr">
         <is>
           <t>Visit types offered: OPD Visit, ER Visit, IPD Visit, Telehealth</t>
         </is>
       </c>
-      <c r="E11" s="799" t="inlineStr">
+      <c r="G11" s="802" t="n"/>
+      <c r="H11" s="802" t="inlineStr">
         <is>
           <t>Mental Health Counselor</t>
         </is>
       </c>
-      <c r="G11" s="799" t="n"/>
+      <c r="I11" s="802" t="n"/>
+      <c r="J11" s="802" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="K11" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L11" s="802" t="n"/>
+      <c r="M11" s="802" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="799" t="inlineStr">
+      <c r="A12" s="802" t="inlineStr">
         <is>
           <t>VISIT-2</t>
         </is>
       </c>
-      <c r="B12" s="799" t="inlineStr">
+      <c r="B12" s="802" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="C12" s="802" t="inlineStr">
+        <is>
+          <t>Mosul</t>
+        </is>
+      </c>
+      <c r="D12" s="802" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
+      <c r="E12" s="802" t="inlineStr">
         <is>
           <t>Leave an OPD or Telehealth visit open</t>
         </is>
       </c>
-      <c r="C12" s="799" t="inlineStr">
+      <c r="F12" s="802" t="inlineStr">
         <is>
           <t>The visit is closed automatically</t>
         </is>
       </c>
-      <c r="E12" s="799" t="inlineStr">
+      <c r="G12" s="802" t="n"/>
+      <c r="H12" s="802" t="inlineStr">
         <is>
           <t>Automatic</t>
         </is>
       </c>
-      <c r="G12" s="799" t="n"/>
+      <c r="I12" s="802" t="n"/>
+      <c r="J12" s="802" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="K12" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L12" s="802" t="n"/>
+      <c r="M12" s="802" t="inlineStr">
+        <is>
+          <t>Auto-close list also names « Home Visit », not a Mosul visit type</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="799" t="inlineStr">
+      <c r="A13" s="802" t="inlineStr">
         <is>
           <t>EDIT-1</t>
         </is>
       </c>
-      <c r="B13" s="799" t="inlineStr">
+      <c r="B13" s="802" t="inlineStr">
+        <is>
+          <t>Patient chart</t>
+        </is>
+      </c>
+      <c r="C13" s="802" t="inlineStr">
+        <is>
+          <t>Mosul</t>
+        </is>
+      </c>
+      <c r="D13" s="802" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
+      <c r="E13" s="802" t="inlineStr">
         <is>
           <t>Edit a form saved more than 24 hours ago</t>
         </is>
       </c>
-      <c r="C13" s="799" t="inlineStr">
+      <c r="F13" s="802" t="inlineStr">
         <is>
           <t>The form can no longer be edited</t>
         </is>
       </c>
-      <c r="E13" s="799" t="inlineStr">
+      <c r="G13" s="802" t="n"/>
+      <c r="H13" s="802" t="inlineStr">
         <is>
           <t>Mental Health Counselor</t>
         </is>
       </c>
+      <c r="I13" s="802" t="n"/>
+      <c r="J13" s="802" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="K13" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L13" s="802" t="n"/>
+      <c r="M13" s="802" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="799" t="inlineStr">
+      <c r="A14" s="802" t="inlineStr">
         <is>
           <t>RDE-1</t>
         </is>
       </c>
-      <c r="B14" s="799" t="inlineStr">
+      <c r="B14" s="802" t="inlineStr">
+        <is>
+          <t>Patient chart</t>
+        </is>
+      </c>
+      <c r="C14" s="802" t="inlineStr">
+        <is>
+          <t>Mosul</t>
+        </is>
+      </c>
+      <c r="D14" s="802" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
+      <c r="E14" s="802" t="inlineStr">
         <is>
           <t>Enter data for a past visit</t>
         </is>
       </c>
-      <c r="C14" s="799" t="inlineStr">
+      <c r="F14" s="802" t="inlineStr">
         <is>
           <t>Retrospective data entry is available</t>
         </is>
       </c>
-      <c r="E14" s="799" t="inlineStr">
+      <c r="G14" s="802" t="n"/>
+      <c r="H14" s="802" t="inlineStr">
         <is>
           <t>Mental Health Counselor</t>
         </is>
       </c>
+      <c r="I14" s="802" t="n"/>
+      <c r="J14" s="802" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="K14" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L14" s="802" t="n"/>
+      <c r="M14" s="802" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="799" t="inlineStr">
+      <c r="A15" s="802" t="inlineStr">
         <is>
           <t>DHIS2-1</t>
         </is>
       </c>
-      <c r="B15" s="799" t="inlineStr">
+      <c r="B15" s="802" t="inlineStr">
+        <is>
+          <t>DHIS2 and OpenFn</t>
+        </is>
+      </c>
+      <c r="C15" s="802" t="inlineStr">
+        <is>
+          <t>Mosul</t>
+        </is>
+      </c>
+      <c r="D15" s="802" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
+      <c r="E15" s="802" t="inlineStr">
         <is>
           <t>Save an F31 mhGAP Baseline with a PHQ-9 score</t>
         </is>
       </c>
-      <c r="C15" s="799" t="inlineStr">
+      <c r="F15" s="802" t="inlineStr">
         <is>
           <t>After the daily sync (17:00), the PHQ-9 score is in DHIS2</t>
         </is>
       </c>
-      <c r="E15" s="799" t="inlineStr">
+      <c r="G15" s="802" t="n"/>
+      <c r="H15" s="802" t="inlineStr">
         <is>
           <t>Automatic</t>
         </is>
       </c>
+      <c r="I15" s="802" t="n"/>
+      <c r="J15" s="802" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K15" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L15" s="802" t="n"/>
+      <c r="M15" s="802" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="802" t="inlineStr">
+        <is>
+          <t>ROLES-1</t>
+        </is>
+      </c>
+      <c r="B16" s="802" t="inlineStr">
+        <is>
+          <t>Access and roles</t>
+        </is>
+      </c>
+      <c r="C16" s="802" t="inlineStr">
+        <is>
+          <t>Matsapha</t>
+        </is>
+      </c>
+      <c r="D16" s="802" t="n"/>
+      <c r="E16" s="802" t="inlineStr">
+        <is>
+          <t>Delete an encounter of a patient</t>
+        </is>
+      </c>
+      <c r="F16" s="802" t="inlineStr">
+        <is>
+          <t>Deletion works</t>
+        </is>
+      </c>
+      <c r="G16" s="802" t="inlineStr">
+        <is>
+          <t>Fictitious patient</t>
+        </is>
+      </c>
+      <c r="H16" s="802" t="inlineStr">
+        <is>
+          <t>Matsapha: Registration Supervisor</t>
+        </is>
+      </c>
+      <c r="I16" s="802" t="inlineStr">
+        <is>
+          <t>Delete Encounters</t>
+        </is>
+      </c>
+      <c r="J16" s="802" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K16" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L16" s="802" t="n"/>
+      <c r="M16" s="802" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="802" t="inlineStr">
+        <is>
+          <t>ROLES-2</t>
+        </is>
+      </c>
+      <c r="B17" s="802" t="inlineStr">
+        <is>
+          <t>Access and roles</t>
+        </is>
+      </c>
+      <c r="C17" s="802" t="inlineStr">
+        <is>
+          <t>Matsapha</t>
+        </is>
+      </c>
+      <c r="D17" s="802" t="n"/>
+      <c r="E17" s="802" t="inlineStr">
+        <is>
+          <t>Open the same patient and look for « Delete »</t>
+        </is>
+      </c>
+      <c r="F17" s="802" t="inlineStr">
+        <is>
+          <t>No delete option</t>
+        </is>
+      </c>
+      <c r="G17" s="802" t="n"/>
+      <c r="H17" s="802" t="inlineStr">
+        <is>
+          <t>Matsapha: Clinical</t>
+        </is>
+      </c>
+      <c r="I17" s="802" t="inlineStr">
+        <is>
+          <t>No Delete Encounters</t>
+        </is>
+      </c>
+      <c r="J17" s="802" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K17" s="802" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="L17" s="802" t="n"/>
+      <c r="M17" s="802" t="n"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <autoFilter ref="A1:M1000"/>
+  <conditionalFormatting sqref="K2:K1000">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="518">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="519">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="520">
+      <formula>"Blocked"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="5">
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Login,Language,Registration,Access and roles,Appointments,Visits,Patient chart,Forms,Orders and lab,DHIS2 and OpenFn,Reports,Printing,Offline"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"All sites,Mosul,Matsapha,Bunia"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Release 1,Release 2,Release 3"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Critical,Normal"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not run,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -13100,6 +13716,7 @@
       <c r="C28" s="238" t="n"/>
       <c r="D28" s="238" t="n"/>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="800" t="inlineStr">
         <is>
@@ -13108,7 +13725,7 @@
       </c>
       <c r="B30" s="799" t="inlineStr">
         <is>
-          <t>Other tests on a question: in 'Comments', 'Test: &lt;what I do&gt; -&gt; &lt;what I should see&gt;'. Tests across questions or forms: 'User flow template' (Action = what I do, Description = what I should see).</t>
+          <t>Other tests on a question: in 'Comments', 'Test: &lt;what I do&gt; -&gt; &lt;what I should see&gt;'. Tests across questions, forms or sites: one row in 'User flow template'. Site = All sites or one site; Release = phase; Result and Tested on are filled when the test is run.</t>
         </is>
       </c>
       <c r="C30" s="799" t="inlineStr">

</xml_diff>